<commit_message>
Fix duplicate ProductID crash and update catalogue Excel files
- Handle duplicate ProductIDs with drop_duplicates(keep='last') before
  set_index().to_dict(), fixing ValueError on Streamlit Cloud
- Update Hem catalogue.xlsx and SacredElement.xlsx with latest data

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SacredElement.xlsx
+++ b/SacredElement.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee11846ce882123f/Desktop/hem-catalogue-app_final-1/hem-catalogue-app-1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Jitesh\Desktop\hem-catalogue-app_final-1\hem-catalogue-app-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{E9A0F783-2FE4-4FED-A298-A23D9B27E370}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24A464F7-83AC-4A6C-861B-8086A2E0DF7F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FF1A79-DA0B-4CF5-914D-3766A2DADD05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DBC07F3F-378B-484D-90AD-F709C710C6B9}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$E$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="176">
   <si>
     <t>Category</t>
   </si>
@@ -50,30 +50,6 @@
     <t>ItemName</t>
   </si>
   <si>
-    <t>Benzoin Resin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Copal Resin </t>
-  </si>
-  <si>
-    <t>Damar Resin</t>
-  </si>
-  <si>
-    <t>Frankincense Resin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Myrrh Resin </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pontifical Resin </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dragons Blood Resin </t>
-  </si>
-  <si>
-    <t>Resin</t>
-  </si>
-  <si>
     <t>Smudge Organic Disc</t>
   </si>
   <si>
@@ -497,18 +473,6 @@
     <t>SH Palo Santo Organic Cones-Shantala</t>
   </si>
   <si>
-    <t>Copal Resin</t>
-  </si>
-  <si>
-    <t>Myrrh Resin</t>
-  </si>
-  <si>
-    <t>Pontifical Resin</t>
-  </si>
-  <si>
-    <t>Dragons Blood Resin</t>
-  </si>
-  <si>
     <t>CONES SACRED ELEMENT ORGANIC</t>
   </si>
   <si>
@@ -527,12 +491,6 @@
     <t xml:space="preserve">Citrus Herbal </t>
   </si>
   <si>
-    <t>sweet rose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JASMINE AND PEACH </t>
-  </si>
-  <si>
     <t>Clay Incense Burner</t>
   </si>
   <si>
@@ -584,25 +542,31 @@
     <t>New Beginnings candle</t>
   </si>
   <si>
-    <t>SELF LOVE INCENSE</t>
-  </si>
-  <si>
-    <t>LOVE POTION INCENSE</t>
-  </si>
-  <si>
-    <t>GROUNDING INCENSE</t>
-  </si>
-  <si>
-    <t>NEW BEGINNINGS INCENSE</t>
-  </si>
-  <si>
-    <t>ENERGY CLEANSE INCENSE</t>
-  </si>
-  <si>
-    <t>ABUNDANCE INCENSE</t>
-  </si>
-  <si>
     <t>Lavender and White Sage Room Spray</t>
+  </si>
+  <si>
+    <t>Sweet Rose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jasmine And Peach </t>
+  </si>
+  <si>
+    <t>Self Love Incense</t>
+  </si>
+  <si>
+    <t>Abundance Incense</t>
+  </si>
+  <si>
+    <t>Energy Cleanse Incense</t>
+  </si>
+  <si>
+    <t>Love Potion incense</t>
+  </si>
+  <si>
+    <t>Grounding incense</t>
+  </si>
+  <si>
+    <t>New Beginnings incense</t>
   </si>
 </sst>
 </file>
@@ -679,7 +643,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -702,6 +666,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -714,7 +691,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -749,6 +726,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,10 +751,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1091,7 +1070,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60D7FE7C-11EF-4516-9D9A-706DE80968F0}">
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="12.453125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="45.453125" style="2" bestFit="1" customWidth="1"/>
@@ -1113,10 +1092,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F1" s="8"/>
       <c r="G1" s="8"/>
@@ -1124,1022 +1103,945 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>164</v>
+        <v>150</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>166</v>
+        <v>152</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>168</v>
+        <v>154</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>170</v>
+        <v>156</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>185</v>
+        <v>20</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>172</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>186</v>
+        <v>20</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>171</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>177</v>
+        <v>163</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>180</v>
+        <v>166</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>171</v>
+        <v>157</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>172</v>
+        <v>158</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>173</v>
+        <v>159</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>174</v>
+        <v>160</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D83" s="2" t="s">
-        <v>3</v>
+        <v>146</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>5</v>
+        <v>148</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>6</v>
+        <v>149</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>10</v>
+        <v>145</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A94" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A95" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E95" xr:uid="{60D7FE7C-11EF-4516-9D9A-706DE80968F0}"/>
+  <autoFilter ref="A1:E88" xr:uid="{60D7FE7C-11EF-4516-9D9A-706DE80968F0}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>